<commit_message>
feat(export): add export button and update template
add export button and update template
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-compare-template.xlsx
+++ b/packages/api-server/assets/evaluation-compare-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8239E3F-F19B-49E5-9351-F78FDDD43019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66891C56-3B9D-4F7A-A0A8-370445E69BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -391,10 +391,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>&lt;%forCell list,i in _data_.scorecards%&gt;&lt;%=list.ciiBestPractice%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.license%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -504,6 +500,10 @@
   </si>
   <si>
     <t>包大小(B)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.ciiBestPractices%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -672,6 +672,15 @@
     <xf numFmtId="179" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -679,15 +688,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1029,14 +1029,14 @@
         <v>3</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="16" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1049,8 +1049,8 @@
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="18"/>
-      <c r="B3" s="14"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="17"/>
       <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1060,8 +1060,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="18"/>
-      <c r="B4" s="14"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="17"/>
       <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
@@ -1071,8 +1071,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="18"/>
-      <c r="B5" s="14"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="17"/>
       <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
@@ -1082,8 +1082,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="18"/>
-      <c r="B6" s="14"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
@@ -1093,8 +1093,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="18"/>
-      <c r="B7" s="14"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
@@ -1104,8 +1104,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="18"/>
-      <c r="B8" s="14"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="3" t="s">
         <v>12</v>
       </c>
@@ -1115,8 +1115,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="18"/>
-      <c r="B9" s="14"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="3" t="s">
         <v>13</v>
       </c>
@@ -1126,8 +1126,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="17"/>
-      <c r="B10" s="15"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
@@ -1137,10 +1137,10 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1154,19 +1154,19 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="18"/>
-      <c r="B12" s="14"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="3" t="s">
         <v>92</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="17"/>
-      <c r="B13" s="15"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="18"/>
       <c r="C13" s="3" t="s">
         <v>19</v>
       </c>
@@ -1178,10 +1178,10 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="16" t="s">
         <v>90</v>
       </c>
       <c r="C14" s="8" t="s">
@@ -1195,8 +1195,8 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="18"/>
-      <c r="B15" s="14"/>
+      <c r="A15" s="15"/>
+      <c r="B15" s="17"/>
       <c r="C15" s="3" t="s">
         <v>22</v>
       </c>
@@ -1208,8 +1208,8 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="18"/>
-      <c r="B16" s="14"/>
+      <c r="A16" s="15"/>
+      <c r="B16" s="17"/>
       <c r="C16" s="3" t="s">
         <v>24</v>
       </c>
@@ -1221,8 +1221,8 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="18"/>
-      <c r="B17" s="14"/>
+      <c r="A17" s="15"/>
+      <c r="B17" s="17"/>
       <c r="C17" s="3" t="s">
         <v>26</v>
       </c>
@@ -1230,12 +1230,12 @@
         <v>25</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>110</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="18"/>
-      <c r="B18" s="14"/>
+      <c r="A18" s="15"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="3" t="s">
         <v>14</v>
       </c>
@@ -1243,12 +1243,12 @@
         <v>27</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="18"/>
-      <c r="B19" s="14"/>
+      <c r="A19" s="15"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="3" t="s">
         <v>29</v>
       </c>
@@ -1256,12 +1256,12 @@
         <v>28</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="18"/>
-      <c r="B20" s="14"/>
+      <c r="A20" s="15"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="3" t="s">
         <v>31</v>
       </c>
@@ -1269,12 +1269,12 @@
         <v>30</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="18"/>
-      <c r="B21" s="14"/>
+      <c r="A21" s="15"/>
+      <c r="B21" s="17"/>
       <c r="C21" s="3" t="s">
         <v>33</v>
       </c>
@@ -1282,12 +1282,12 @@
         <v>32</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="18"/>
-      <c r="B22" s="14"/>
+      <c r="A22" s="15"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="3" t="s">
         <v>35</v>
       </c>
@@ -1295,12 +1295,12 @@
         <v>34</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="18"/>
-      <c r="B23" s="14"/>
+      <c r="A23" s="15"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="3" t="s">
         <v>36</v>
       </c>
@@ -1308,12 +1308,12 @@
         <v>68</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="18"/>
-      <c r="B24" s="14"/>
+      <c r="A24" s="15"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="3" t="s">
         <v>38</v>
       </c>
@@ -1321,12 +1321,12 @@
         <v>37</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="18"/>
-      <c r="B25" s="14"/>
+      <c r="A25" s="15"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="3" t="s">
         <v>40</v>
       </c>
@@ -1334,12 +1334,12 @@
         <v>39</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="18"/>
-      <c r="B26" s="14"/>
+      <c r="A26" s="15"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="3" t="s">
         <v>42</v>
       </c>
@@ -1347,12 +1347,12 @@
         <v>41</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="18"/>
-      <c r="B27" s="15"/>
+      <c r="A27" s="15"/>
+      <c r="B27" s="18"/>
       <c r="C27" s="3" t="s">
         <v>44</v>
       </c>
@@ -1360,12 +1360,12 @@
         <v>43</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="18"/>
-      <c r="B28" s="13" t="s">
+      <c r="A28" s="15"/>
+      <c r="B28" s="16" t="s">
         <v>45</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -1375,12 +1375,12 @@
         <v>74</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="18"/>
-      <c r="B29" s="14"/>
+      <c r="A29" s="15"/>
+      <c r="B29" s="17"/>
       <c r="C29" s="3" t="s">
         <v>47</v>
       </c>
@@ -1388,12 +1388,12 @@
         <v>75</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="18"/>
-      <c r="B30" s="14"/>
+      <c r="A30" s="15"/>
+      <c r="B30" s="17"/>
       <c r="C30" s="3" t="s">
         <v>48</v>
       </c>
@@ -1401,12 +1401,12 @@
         <v>76</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="17"/>
-      <c r="B31" s="15"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="18"/>
       <c r="C31" s="3" t="s">
         <v>49</v>
       </c>
@@ -1414,11 +1414,11 @@
         <v>77</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="13" t="s">
         <v>50</v>
       </c>
       <c r="B32" s="5" t="s">
@@ -1433,23 +1433,23 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="17"/>
+      <c r="A33" s="14"/>
       <c r="B33" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="16" t="s">
         <v>55</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -1457,12 +1457,12 @@
       </c>
       <c r="D34" s="4"/>
       <c r="E34" s="12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="18"/>
-      <c r="B35" s="14"/>
+      <c r="A35" s="15"/>
+      <c r="B35" s="17"/>
       <c r="C35" s="3" t="s">
         <v>56</v>
       </c>
@@ -1472,8 +1472,8 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="18"/>
-      <c r="B36" s="14"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="17"/>
       <c r="C36" s="3" t="s">
         <v>57</v>
       </c>
@@ -1483,8 +1483,8 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="18"/>
-      <c r="B37" s="15"/>
+      <c r="A37" s="15"/>
+      <c r="B37" s="18"/>
       <c r="C37" s="3" t="s">
         <v>59</v>
       </c>
@@ -1492,12 +1492,12 @@
         <v>58</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="18"/>
-      <c r="B38" s="13" t="s">
+      <c r="A38" s="15"/>
+      <c r="B38" s="16" t="s">
         <v>61</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -1507,12 +1507,12 @@
         <v>60</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="18"/>
-      <c r="B39" s="14"/>
+      <c r="A39" s="15"/>
+      <c r="B39" s="17"/>
       <c r="C39" s="3" t="s">
         <v>64</v>
       </c>
@@ -1520,12 +1520,12 @@
         <v>63</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="18"/>
-      <c r="B40" s="14"/>
+      <c r="A40" s="15"/>
+      <c r="B40" s="17"/>
       <c r="C40" s="3" t="s">
         <v>78</v>
       </c>
@@ -1537,8 +1537,8 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="18"/>
-      <c r="B41" s="15"/>
+      <c r="A41" s="15"/>
+      <c r="B41" s="18"/>
       <c r="C41" s="3" t="s">
         <v>80</v>
       </c>
@@ -1550,8 +1550,8 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="18"/>
-      <c r="B42" s="13" t="s">
+      <c r="A42" s="15"/>
+      <c r="B42" s="16" t="s">
         <v>65</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -1561,12 +1561,12 @@
         <v>82</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="18"/>
-      <c r="B43" s="14"/>
+      <c r="A43" s="15"/>
+      <c r="B43" s="17"/>
       <c r="C43" s="3" t="s">
         <v>66</v>
       </c>
@@ -1574,12 +1574,12 @@
         <v>83</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="18"/>
-      <c r="B44" s="14"/>
+      <c r="A44" s="15"/>
+      <c r="B44" s="17"/>
       <c r="C44" s="3" t="s">
         <v>71</v>
       </c>
@@ -1587,12 +1587,12 @@
         <v>84</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="18"/>
-      <c r="B45" s="14"/>
+      <c r="A45" s="15"/>
+      <c r="B45" s="17"/>
       <c r="C45" s="3" t="s">
         <v>88</v>
       </c>
@@ -1600,12 +1600,12 @@
         <v>89</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="18"/>
-      <c r="B46" s="14"/>
+      <c r="A46" s="15"/>
+      <c r="B46" s="17"/>
       <c r="C46" s="3" t="s">
         <v>87</v>
       </c>
@@ -1613,12 +1613,12 @@
         <v>85</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="17"/>
-      <c r="B47" s="15"/>
+      <c r="A47" s="14"/>
+      <c r="B47" s="18"/>
       <c r="C47" s="3" t="s">
         <v>67</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>86</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1636,13 +1636,13 @@
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="B28:B31"/>
+    <mergeCell ref="A14:A31"/>
+    <mergeCell ref="B14:B27"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="A34:A47"/>
     <mergeCell ref="B34:B37"/>
     <mergeCell ref="B38:B41"/>
     <mergeCell ref="B42:B47"/>
-    <mergeCell ref="A14:A31"/>
-    <mergeCell ref="B14:B27"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(export): update export template
update export template
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-compare-template.xlsx
+++ b/packages/api-server/assets/evaluation-compare-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A777143-5F06-47EC-A881-74991844D1CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E6C716-6B03-44D4-A8E9-329288C0AF3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="143">
   <si>
     <t>维度</t>
   </si>
@@ -345,124 +345,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>&lt;%forCell list,i in _data_.contributors%&gt;&lt;%=list%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.dependentRepositories%&gt;&lt;%=list%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.star%&gt;&lt;%=list%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.star%&gt;&lt;%=list%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.fork%&gt;&lt;%=list%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.score%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.document%&gt;&lt;%=list.documentScore%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.codeReview%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.maintained%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.license%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.securityPolicy%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.dangerousWorkflow%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.tokenPermissions%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.branchProtection%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.fuzzing%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.sast%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.vulnerabilities%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.pinnedDependencies%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.busFactor%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.openrank%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.criticalityScore%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.orgCount%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.commentFrequency%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.updatedIssuesCount%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.closedIssuesCount%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.recentReleasesCount%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation %&gt;&lt;%=list.npmDownloads/1000%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.commitFrequency%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.codeLines%&gt;&lt;%=list/1000%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.binaryArtifacts%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>&lt;%forCell list,i in _data_?.sonarCloudScan%&gt;&lt;%=list?.securityReviewRating || 'N/A' %&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -483,18 +365,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>&lt;%forCell list,i in _data_?.gzipSize%&gt;&lt;%=list%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>包大小(B)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%=list.ciiBestPractices%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>功能</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -515,19 +389,143 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.functionScore%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.qualityScore%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.ecologyScore%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%=list.performanceScore%&gt;</t>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.functionScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.performanceScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.qualityScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.ecologyScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.codeLines%&gt;&lt;%~list/1000%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.document%&gt;&lt;%~list.documentScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_?.gzipSize%&gt;&lt;%~list%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.score%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.codeReview%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.maintained%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.ciiBestPractices%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.license%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.securityPolicy%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.dangerousWorkflow%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.branchProtection%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.tokenPermissions%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.binaryArtifacts%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.fuzzing%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.sast%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.vulnerabilities%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.pinnedDependencies%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation %&gt;&lt;%~list.npmDownloads/1000%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.star%&gt;&lt;%~list%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.fork%&gt;&lt;%~list%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.busFactor%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.openrank%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.criticalityScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.contributors%&gt;&lt;%~list%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.dependentRepositories%&gt;&lt;%~list%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.commitFrequency%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.orgCount%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.commentFrequency%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.updatedIssuesCount%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.closedIssuesCount%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.recentReleasesCount%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -699,9 +697,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -709,6 +704,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1053,14 +1051,14 @@
         <v>3</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="15" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1073,8 +1071,8 @@
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="15"/>
-      <c r="B3" s="17"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1084,8 +1082,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="15"/>
-      <c r="B4" s="17"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
@@ -1095,8 +1093,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="B5" s="17"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
@@ -1106,30 +1104,30 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="15"/>
-      <c r="B6" s="17"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="11" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="15"/>
-      <c r="B7" s="17"/>
+      <c r="A7" s="14"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="11" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="15"/>
-      <c r="B8" s="17"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="3" t="s">
         <v>12</v>
       </c>
@@ -1139,8 +1137,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="15"/>
-      <c r="B9" s="17"/>
+      <c r="A9" s="14"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="3" t="s">
         <v>13</v>
       </c>
@@ -1150,65 +1148,65 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="15"/>
-      <c r="B10" s="17"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="16"/>
       <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="5" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="15"/>
-      <c r="B11" s="17"/>
+      <c r="A11" s="14"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="3" t="s">
-        <v>135</v>
+        <v>103</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="5" t="s">
-        <v>140</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="15"/>
-      <c r="B12" s="17"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="3" t="s">
-        <v>137</v>
+        <v>105</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="5" t="s">
-        <v>143</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="15"/>
-      <c r="B13" s="17"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="3" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="5" t="s">
-        <v>141</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="15"/>
-      <c r="B14" s="17"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="3" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="5" t="s">
-        <v>142</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="B15" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>15</v>
       </c>
       <c r="C15" s="3" t="s">
@@ -1222,18 +1220,18 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="15"/>
-      <c r="B16" s="17"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="16"/>
       <c r="C16" s="3" t="s">
         <v>89</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="6" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="14"/>
+      <c r="A17" s="17"/>
       <c r="B17" s="18"/>
       <c r="C17" s="3" t="s">
         <v>18</v>
@@ -1242,7 +1240,7 @@
         <v>17</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1261,23 +1259,23 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="14"/>
+      <c r="A19" s="17"/>
       <c r="B19" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>133</v>
+        <v>102</v>
       </c>
       <c r="D19" s="4"/>
       <c r="E19" s="12" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="B20" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="B20" s="15" t="s">
         <v>87</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -1287,12 +1285,12 @@
         <v>70</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="15"/>
-      <c r="B21" s="17"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="3" t="s">
         <v>20</v>
       </c>
@@ -1300,12 +1298,12 @@
         <v>19</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="15"/>
-      <c r="B22" s="17"/>
+      <c r="A22" s="14"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="3" t="s">
         <v>22</v>
       </c>
@@ -1313,12 +1311,12 @@
         <v>21</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="15"/>
-      <c r="B23" s="17"/>
+      <c r="A23" s="14"/>
+      <c r="B23" s="16"/>
       <c r="C23" s="3" t="s">
         <v>24</v>
       </c>
@@ -1326,12 +1324,12 @@
         <v>23</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="15"/>
-      <c r="B24" s="17"/>
+      <c r="A24" s="14"/>
+      <c r="B24" s="16"/>
       <c r="C24" s="3" t="s">
         <v>14</v>
       </c>
@@ -1339,12 +1337,12 @@
         <v>25</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="15"/>
-      <c r="B25" s="17"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="3" t="s">
         <v>27</v>
       </c>
@@ -1352,12 +1350,12 @@
         <v>26</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="15"/>
-      <c r="B26" s="17"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="3" t="s">
         <v>29</v>
       </c>
@@ -1365,12 +1363,12 @@
         <v>28</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="15"/>
-      <c r="B27" s="17"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="16"/>
       <c r="C27" s="3" t="s">
         <v>31</v>
       </c>
@@ -1378,12 +1376,12 @@
         <v>30</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="15"/>
-      <c r="B28" s="17"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="16"/>
       <c r="C28" s="3" t="s">
         <v>33</v>
       </c>
@@ -1391,12 +1389,12 @@
         <v>32</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="15"/>
-      <c r="B29" s="17"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="16"/>
       <c r="C29" s="3" t="s">
         <v>34</v>
       </c>
@@ -1404,12 +1402,12 @@
         <v>65</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="15"/>
-      <c r="B30" s="17"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="16"/>
       <c r="C30" s="3" t="s">
         <v>36</v>
       </c>
@@ -1417,12 +1415,12 @@
         <v>35</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="15"/>
-      <c r="B31" s="17"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="16"/>
       <c r="C31" s="3" t="s">
         <v>38</v>
       </c>
@@ -1430,12 +1428,12 @@
         <v>37</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="15"/>
-      <c r="B32" s="17"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="16"/>
       <c r="C32" s="3" t="s">
         <v>40</v>
       </c>
@@ -1443,11 +1441,11 @@
         <v>39</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="15"/>
+      <c r="A33" s="14"/>
       <c r="B33" s="18"/>
       <c r="C33" s="3" t="s">
         <v>42</v>
@@ -1456,12 +1454,12 @@
         <v>41</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="15"/>
-      <c r="B34" s="16" t="s">
+      <c r="A34" s="14"/>
+      <c r="B34" s="15" t="s">
         <v>43</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -1471,12 +1469,12 @@
         <v>71</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>130</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="15"/>
-      <c r="B35" s="17"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="16"/>
       <c r="C35" s="3" t="s">
         <v>45</v>
       </c>
@@ -1484,12 +1482,12 @@
         <v>72</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>129</v>
+        <v>99</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="15"/>
-      <c r="B36" s="17"/>
+      <c r="A36" s="14"/>
+      <c r="B36" s="16"/>
       <c r="C36" s="3" t="s">
         <v>46</v>
       </c>
@@ -1497,11 +1495,11 @@
         <v>73</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>128</v>
+        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="14"/>
+      <c r="A37" s="17"/>
       <c r="B37" s="18"/>
       <c r="C37" s="3" t="s">
         <v>47</v>
@@ -1510,14 +1508,14 @@
         <v>74</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>127</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B38" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="B38" s="15" t="s">
         <v>52</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -1525,33 +1523,33 @@
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="12" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="15"/>
-      <c r="B39" s="17"/>
+      <c r="A39" s="14"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="11" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="15"/>
-      <c r="B40" s="17"/>
+      <c r="A40" s="14"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D40" s="7"/>
       <c r="E40" s="11" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="15"/>
+      <c r="A41" s="14"/>
       <c r="B41" s="18"/>
       <c r="C41" s="3" t="s">
         <v>56</v>
@@ -1560,12 +1558,12 @@
         <v>55</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="15"/>
-      <c r="B42" s="16" t="s">
+      <c r="A42" s="14"/>
+      <c r="B42" s="15" t="s">
         <v>58</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -1575,12 +1573,12 @@
         <v>57</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="15"/>
-      <c r="B43" s="17"/>
+      <c r="A43" s="14"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="3" t="s">
         <v>61</v>
       </c>
@@ -1588,12 +1586,12 @@
         <v>60</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="15"/>
-      <c r="B44" s="17"/>
+      <c r="A44" s="14"/>
+      <c r="B44" s="16"/>
       <c r="C44" s="3" t="s">
         <v>75</v>
       </c>
@@ -1601,11 +1599,11 @@
         <v>76</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>97</v>
+        <v>135</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="15"/>
+      <c r="A45" s="14"/>
       <c r="B45" s="18"/>
       <c r="C45" s="3" t="s">
         <v>77</v>
@@ -1614,12 +1612,12 @@
         <v>78</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>98</v>
+        <v>136</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="15"/>
-      <c r="B46" s="16" t="s">
+      <c r="A46" s="14"/>
+      <c r="B46" s="15" t="s">
         <v>62</v>
       </c>
       <c r="C46" s="3" t="s">
@@ -1629,12 +1627,12 @@
         <v>79</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="15"/>
-      <c r="B47" s="17"/>
+      <c r="A47" s="14"/>
+      <c r="B47" s="16"/>
       <c r="C47" s="3" t="s">
         <v>63</v>
       </c>
@@ -1642,12 +1640,12 @@
         <v>80</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="15"/>
-      <c r="B48" s="17"/>
+      <c r="A48" s="14"/>
+      <c r="B48" s="16"/>
       <c r="C48" s="3" t="s">
         <v>68</v>
       </c>
@@ -1655,12 +1653,12 @@
         <v>81</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>119</v>
+        <v>139</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="15"/>
-      <c r="B49" s="17"/>
+      <c r="A49" s="14"/>
+      <c r="B49" s="16"/>
       <c r="C49" s="3" t="s">
         <v>85</v>
       </c>
@@ -1668,12 +1666,12 @@
         <v>86</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>120</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="15"/>
-      <c r="B50" s="17"/>
+      <c r="A50" s="14"/>
+      <c r="B50" s="16"/>
       <c r="C50" s="3" t="s">
         <v>84</v>
       </c>
@@ -1681,11 +1679,11 @@
         <v>82</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="14"/>
+      <c r="A51" s="17"/>
       <c r="B51" s="18"/>
       <c r="C51" s="3" t="s">
         <v>64</v>
@@ -1694,11 +1692,15 @@
         <v>83</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>122</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A38:A51"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="B46:B51"/>
     <mergeCell ref="A2:A14"/>
     <mergeCell ref="B2:B14"/>
     <mergeCell ref="A15:A17"/>
@@ -1707,10 +1709,6 @@
     <mergeCell ref="A20:A37"/>
     <mergeCell ref="B20:B33"/>
     <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A38:A51"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="B46:B51"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(export): add field innovationScore in template
add field innovationScore in template
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-compare-template.xlsx
+++ b/packages/api-server/assets/evaluation-compare-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C79A6DA-E8A8-4BD8-A897-7F79D9BFCEAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A94304-72C4-4378-B6FB-B72657BFDE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="146">
   <si>
     <t>维度</t>
   </si>
@@ -533,6 +533,14 @@
   </si>
   <si>
     <t>&lt;%=_data_.title%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>创新</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.innovationScore%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -608,7 +616,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -668,13 +676,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -708,19 +753,37 @@
     <xf numFmtId="179" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1037,7 +1100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.375" style="1" customWidth="1"/>
@@ -1049,13 +1112,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="15"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
@@ -1075,10 +1138,10 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -1090,8 +1153,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="11"/>
-      <c r="B4" s="12"/>
+      <c r="A4" s="17"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
@@ -1101,8 +1164,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="11"/>
-      <c r="B5" s="12"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="3" t="s">
         <v>6</v>
       </c>
@@ -1112,8 +1175,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="3" t="s">
         <v>7</v>
       </c>
@@ -1123,8 +1186,8 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
@@ -1134,8 +1197,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="20"/>
       <c r="C8" s="3" t="s">
         <v>9</v>
       </c>
@@ -1145,8 +1208,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="3" t="s">
         <v>10</v>
       </c>
@@ -1156,8 +1219,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="20"/>
       <c r="C10" s="3" t="s">
         <v>11</v>
       </c>
@@ -1167,8 +1230,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="3" t="s">
         <v>99</v>
       </c>
@@ -1180,8 +1243,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="3" t="s">
         <v>101</v>
       </c>
@@ -1193,8 +1256,8 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="3" t="s">
         <v>100</v>
       </c>
@@ -1206,8 +1269,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="B14" s="12"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="20"/>
       <c r="C14" s="3" t="s">
         <v>102</v>
       </c>
@@ -1219,513 +1282,526 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="18"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B16" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="3" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="14"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="4"/>
-      <c r="E16" s="6" t="s">
+      <c r="D17" s="4"/>
+      <c r="E17" s="6" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="3" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B19" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="6" t="s">
+      <c r="D19" s="4"/>
+      <c r="E19" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
-      <c r="B19" s="5" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="14"/>
+      <c r="B20" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C20" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="10" t="s">
+      <c r="D20" s="4"/>
+      <c r="E20" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B21" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="3" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="14"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E22" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="3" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="14"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E23" s="7" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="11"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="3" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="14"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E24" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="11"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="3" t="s">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="14"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D25" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E25" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="11"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="3" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="14"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E26" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="3" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="14"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D27" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E27" s="7" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="3" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="14"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D28" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="E28" s="7" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="11"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="3" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="14"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D29" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E29" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="11"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="3" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="14"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="E30" s="7" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="11"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="3" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="14"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D31" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E31" s="7" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="3" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="14"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D32" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E32" s="7" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="11"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="3" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="14"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="E33" s="7" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="3" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="14"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="E34" s="7" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="14"/>
+      <c r="B35" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C35" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D35" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="11"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="3" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="14"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D36" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E36" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="11"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="3" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="14"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D37" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="E37" s="5" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="11"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="3" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="14"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D38" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="11" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B39" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C39" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D38" s="4"/>
-      <c r="E38" s="10" t="s">
+      <c r="D39" s="4"/>
+      <c r="E39" s="10" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="11"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="3" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="14"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="D39" s="4"/>
-      <c r="E39" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="11"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="14"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D41" s="4"/>
+      <c r="E41" s="9" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="11"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="3" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="14"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D42" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="E42" s="9" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="11"/>
-      <c r="B42" s="12" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="14"/>
+      <c r="B43" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C43" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="D43" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="E43" s="6" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="11"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="3" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="14"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="D44" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="E44" s="6" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="11"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="3" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="14"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D44" s="4" t="s">
+      <c r="D45" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E44" s="9" t="s">
+      <c r="E45" s="9" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="11"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="3" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="14"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="D46" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E45" s="9" t="s">
+      <c r="E46" s="9" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="11"/>
-      <c r="B46" s="12" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="14"/>
+      <c r="B47" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C47" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="4" t="s">
+      <c r="D47" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="E47" s="6" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="11"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="3" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="14"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D47" s="4" t="s">
+      <c r="D48" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="E48" s="6" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="11"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="3" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="14"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D48" s="4" t="s">
+      <c r="D49" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="E49" s="6" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="11"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="3" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="14"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D49" s="4" t="s">
+      <c r="D50" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E50" s="6" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="11"/>
-      <c r="B50" s="12"/>
-      <c r="C50" s="3" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="14"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="D51" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E50" s="6" t="s">
+      <c r="E51" s="6" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="11"/>
-      <c r="B51" s="12"/>
-      <c r="C51" s="3" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="14"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D51" s="4" t="s">
+      <c r="D52" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="E52" s="6" t="s">
         <v>138</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:A14"/>
-    <mergeCell ref="B3:B14"/>
-    <mergeCell ref="A38:A51"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="B46:B51"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="A20:A37"/>
-    <mergeCell ref="B20:B33"/>
-    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A39:A52"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B47:B52"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="A21:A38"/>
+    <mergeCell ref="B21:B34"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A3:A15"/>
+    <mergeCell ref="B3:B15"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: fixed export bug
fixed export bug
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-compare-template.xlsx
+++ b/packages/api-server/assets/evaluation-compare-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A94304-72C4-4378-B6FB-B72657BFDE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA4636F-6C5D-47C6-8A72-2C00C1EF77D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="评估结果" sheetId="1" r:id="rId1"/>
@@ -404,62 +404,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.score%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.codeReview%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.maintained%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.ciiBestPractices%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.license%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.securityPolicy%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.dangerousWorkflow%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.branchProtection%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.tokenPermissions%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.binaryArtifacts%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.fuzzing%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.sast%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.vulnerabilities%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.pinnedDependencies%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>&lt;%forCell list,i in _data_.evaluation %&gt;&lt;%~list.npmDownloads/1000%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -541,6 +485,62 @@
   </si>
   <si>
     <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.innovationScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.score || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.codeReview || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.maintained || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.ciiBestPractices || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.license || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.securityPolicy || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.dangerousWorkflow || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.branchProtection || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.tokenPermissions || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.binaryArtifacts || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.fuzzing || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.sast || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.vulnerabilities || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.pinnedDependencies || 'N/A' %&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1101,31 +1101,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E52"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="24.625" customWidth="1"/>
-    <col min="4" max="4" width="28.875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="28.88671875" style="2" customWidth="1"/>
     <col min="5" max="5" width="62" style="2" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
       <c r="D1" s="12"/>
       <c r="E1" s="13"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>1</v>
@@ -1137,12 +1137,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>4</v>
@@ -1152,7 +1152,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A4" s="17"/>
       <c r="B4" s="20"/>
       <c r="C4" s="3" t="s">
@@ -1163,7 +1163,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="20"/>
       <c r="C5" s="3" t="s">
@@ -1174,7 +1174,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A6" s="17"/>
       <c r="B6" s="20"/>
       <c r="C6" s="3" t="s">
@@ -1182,10 +1182,10 @@
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A7" s="17"/>
       <c r="B7" s="20"/>
       <c r="C7" s="3" t="s">
@@ -1193,10 +1193,10 @@
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="20"/>
       <c r="C8" s="3" t="s">
@@ -1207,7 +1207,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="20"/>
       <c r="C9" s="3" t="s">
@@ -1218,7 +1218,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="20"/>
       <c r="C10" s="3" t="s">
@@ -1229,72 +1229,72 @@
         <v>103</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="20"/>
       <c r="C11" s="3" t="s">
         <v>99</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="20"/>
       <c r="C12" s="3" t="s">
         <v>101</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="20"/>
       <c r="C13" s="3" t="s">
         <v>100</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A14" s="17"/>
       <c r="B14" s="20"/>
       <c r="C14" s="3" t="s">
         <v>102</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A15" s="18"/>
       <c r="B15" s="21"/>
       <c r="C15" s="3" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>99</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A17" s="14"/>
       <c r="B17" s="15"/>
       <c r="C17" s="3" t="s">
@@ -1322,7 +1322,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A18" s="14"/>
       <c r="B18" s="15"/>
       <c r="C18" s="3" t="s">
@@ -1335,7 +1335,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>45</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A20" s="14"/>
       <c r="B20" s="5" t="s">
         <v>48</v>
@@ -1363,7 +1363,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>100</v>
       </c>
@@ -1377,10 +1377,10 @@
         <v>67</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A22" s="14"/>
       <c r="B22" s="15"/>
       <c r="C22" s="3" t="s">
@@ -1390,10 +1390,10 @@
         <v>16</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A23" s="14"/>
       <c r="B23" s="15"/>
       <c r="C23" s="3" t="s">
@@ -1403,10 +1403,10 @@
         <v>18</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A24" s="14"/>
       <c r="B24" s="15"/>
       <c r="C24" s="3" t="s">
@@ -1416,10 +1416,10 @@
         <v>20</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A25" s="14"/>
       <c r="B25" s="15"/>
       <c r="C25" s="3" t="s">
@@ -1429,10 +1429,10 @@
         <v>22</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A26" s="14"/>
       <c r="B26" s="15"/>
       <c r="C26" s="3" t="s">
@@ -1442,10 +1442,10 @@
         <v>23</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A27" s="14"/>
       <c r="B27" s="15"/>
       <c r="C27" s="3" t="s">
@@ -1455,10 +1455,10 @@
         <v>25</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A28" s="14"/>
       <c r="B28" s="15"/>
       <c r="C28" s="3" t="s">
@@ -1468,10 +1468,10 @@
         <v>27</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
       <c r="C29" s="3" t="s">
@@ -1481,10 +1481,10 @@
         <v>29</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
       <c r="C30" s="3" t="s">
@@ -1494,10 +1494,10 @@
         <v>62</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
       <c r="C31" s="3" t="s">
@@ -1507,10 +1507,10 @@
         <v>32</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="15"/>
       <c r="C32" s="3" t="s">
@@ -1520,10 +1520,10 @@
         <v>34</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A33" s="14"/>
       <c r="B33" s="15"/>
       <c r="C33" s="3" t="s">
@@ -1533,10 +1533,10 @@
         <v>36</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A34" s="14"/>
       <c r="B34" s="15"/>
       <c r="C34" s="3" t="s">
@@ -1546,10 +1546,10 @@
         <v>38</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
         <v>40</v>
@@ -1564,7 +1564,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="15"/>
       <c r="C36" s="3" t="s">
@@ -1577,7 +1577,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="15"/>
       <c r="C37" s="3" t="s">
@@ -1590,7 +1590,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
       <c r="B38" s="15"/>
       <c r="C38" s="3" t="s">
@@ -1603,7 +1603,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>102</v>
       </c>
@@ -1615,10 +1615,10 @@
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A40" s="14"/>
       <c r="B40" s="15"/>
       <c r="C40" s="3" t="s">
@@ -1626,10 +1626,10 @@
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A41" s="14"/>
       <c r="B41" s="15"/>
       <c r="C41" s="3" t="s">
@@ -1637,10 +1637,10 @@
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A42" s="14"/>
       <c r="B42" s="15"/>
       <c r="C42" s="3" t="s">
@@ -1650,10 +1650,10 @@
         <v>52</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A43" s="14"/>
       <c r="B43" s="15" t="s">
         <v>55</v>
@@ -1665,10 +1665,10 @@
         <v>54</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
       <c r="B44" s="15"/>
       <c r="C44" s="3" t="s">
@@ -1678,10 +1678,10 @@
         <v>57</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A45" s="14"/>
       <c r="B45" s="15"/>
       <c r="C45" s="3" t="s">
@@ -1691,10 +1691,10 @@
         <v>73</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="15"/>
       <c r="C46" s="3" t="s">
@@ -1704,10 +1704,10 @@
         <v>75</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A47" s="14"/>
       <c r="B47" s="15" t="s">
         <v>59</v>
@@ -1719,10 +1719,10 @@
         <v>76</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A48" s="14"/>
       <c r="B48" s="15"/>
       <c r="C48" s="3" t="s">
@@ -1732,10 +1732,10 @@
         <v>77</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A49" s="14"/>
       <c r="B49" s="15"/>
       <c r="C49" s="3" t="s">
@@ -1745,10 +1745,10 @@
         <v>78</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A50" s="14"/>
       <c r="B50" s="15"/>
       <c r="C50" s="3" t="s">
@@ -1758,10 +1758,10 @@
         <v>83</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A51" s="14"/>
       <c r="B51" s="15"/>
       <c r="C51" s="3" t="s">
@@ -1771,10 +1771,10 @@
         <v>79</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A52" s="14"/>
       <c r="B52" s="15"/>
       <c r="C52" s="3" t="s">
@@ -1784,7 +1784,7 @@
         <v>80</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: fixed export bug (#784)
fixed export bug
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-compare-template.xlsx
+++ b/packages/api-server/assets/evaluation-compare-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A94304-72C4-4378-B6FB-B72657BFDE25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA4636F-6C5D-47C6-8A72-2C00C1EF77D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="评估结果" sheetId="1" r:id="rId1"/>
@@ -404,62 +404,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.score%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.codeReview%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.maintained%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.ciiBestPractices%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.license%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.securityPolicy%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.dangerousWorkflow%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.branchProtection%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.tokenPermissions%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.binaryArtifacts%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.fuzzing%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.sast%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.vulnerabilities%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list.pinnedDependencies%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>&lt;%forCell list,i in _data_.evaluation %&gt;&lt;%~list.npmDownloads/1000%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -541,6 +485,62 @@
   </si>
   <si>
     <t>&lt;%forCell list,i in _data_.evaluation%&gt;&lt;%~list.innovationScore%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.score || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.codeReview || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.maintained || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.ciiBestPractices || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.license || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.securityPolicy || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.dangerousWorkflow || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.branchProtection || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.tokenPermissions || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.binaryArtifacts || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.fuzzing || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.sast || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.vulnerabilities || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%forCell list,i in _data_.scorecard%&gt;&lt;%~list?.pinnedDependencies || 'N/A' %&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1101,31 +1101,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E52"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="24.625" customWidth="1"/>
-    <col min="4" max="4" width="28.875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="28.88671875" style="2" customWidth="1"/>
     <col min="5" max="5" width="62" style="2" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
       <c r="D1" s="12"/>
       <c r="E1" s="13"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>1</v>
@@ -1137,12 +1137,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>4</v>
@@ -1152,7 +1152,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A4" s="17"/>
       <c r="B4" s="20"/>
       <c r="C4" s="3" t="s">
@@ -1163,7 +1163,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="20"/>
       <c r="C5" s="3" t="s">
@@ -1174,7 +1174,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A6" s="17"/>
       <c r="B6" s="20"/>
       <c r="C6" s="3" t="s">
@@ -1182,10 +1182,10 @@
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A7" s="17"/>
       <c r="B7" s="20"/>
       <c r="C7" s="3" t="s">
@@ -1193,10 +1193,10 @@
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="20"/>
       <c r="C8" s="3" t="s">
@@ -1207,7 +1207,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="20"/>
       <c r="C9" s="3" t="s">
@@ -1218,7 +1218,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="20"/>
       <c r="C10" s="3" t="s">
@@ -1229,72 +1229,72 @@
         <v>103</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="20"/>
       <c r="C11" s="3" t="s">
         <v>99</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="20"/>
       <c r="C12" s="3" t="s">
         <v>101</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A13" s="17"/>
       <c r="B13" s="20"/>
       <c r="C13" s="3" t="s">
         <v>100</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A14" s="17"/>
       <c r="B14" s="20"/>
       <c r="C14" s="3" t="s">
         <v>102</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A15" s="18"/>
       <c r="B15" s="21"/>
       <c r="C15" s="3" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>99</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A17" s="14"/>
       <c r="B17" s="15"/>
       <c r="C17" s="3" t="s">
@@ -1322,7 +1322,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A18" s="14"/>
       <c r="B18" s="15"/>
       <c r="C18" s="3" t="s">
@@ -1335,7 +1335,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>45</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A20" s="14"/>
       <c r="B20" s="5" t="s">
         <v>48</v>
@@ -1363,7 +1363,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>100</v>
       </c>
@@ -1377,10 +1377,10 @@
         <v>67</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A22" s="14"/>
       <c r="B22" s="15"/>
       <c r="C22" s="3" t="s">
@@ -1390,10 +1390,10 @@
         <v>16</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A23" s="14"/>
       <c r="B23" s="15"/>
       <c r="C23" s="3" t="s">
@@ -1403,10 +1403,10 @@
         <v>18</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A24" s="14"/>
       <c r="B24" s="15"/>
       <c r="C24" s="3" t="s">
@@ -1416,10 +1416,10 @@
         <v>20</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A25" s="14"/>
       <c r="B25" s="15"/>
       <c r="C25" s="3" t="s">
@@ -1429,10 +1429,10 @@
         <v>22</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A26" s="14"/>
       <c r="B26" s="15"/>
       <c r="C26" s="3" t="s">
@@ -1442,10 +1442,10 @@
         <v>23</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A27" s="14"/>
       <c r="B27" s="15"/>
       <c r="C27" s="3" t="s">
@@ -1455,10 +1455,10 @@
         <v>25</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A28" s="14"/>
       <c r="B28" s="15"/>
       <c r="C28" s="3" t="s">
@@ -1468,10 +1468,10 @@
         <v>27</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
       <c r="C29" s="3" t="s">
@@ -1481,10 +1481,10 @@
         <v>29</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
       <c r="C30" s="3" t="s">
@@ -1494,10 +1494,10 @@
         <v>62</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
       <c r="C31" s="3" t="s">
@@ -1507,10 +1507,10 @@
         <v>32</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="15"/>
       <c r="C32" s="3" t="s">
@@ -1520,10 +1520,10 @@
         <v>34</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A33" s="14"/>
       <c r="B33" s="15"/>
       <c r="C33" s="3" t="s">
@@ -1533,10 +1533,10 @@
         <v>36</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A34" s="14"/>
       <c r="B34" s="15"/>
       <c r="C34" s="3" t="s">
@@ -1546,10 +1546,10 @@
         <v>38</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
       <c r="B35" s="15" t="s">
         <v>40</v>
@@ -1564,7 +1564,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="15"/>
       <c r="C36" s="3" t="s">
@@ -1577,7 +1577,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="15"/>
       <c r="C37" s="3" t="s">
@@ -1590,7 +1590,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
       <c r="B38" s="15"/>
       <c r="C38" s="3" t="s">
@@ -1603,7 +1603,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>102</v>
       </c>
@@ -1615,10 +1615,10 @@
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A40" s="14"/>
       <c r="B40" s="15"/>
       <c r="C40" s="3" t="s">
@@ -1626,10 +1626,10 @@
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A41" s="14"/>
       <c r="B41" s="15"/>
       <c r="C41" s="3" t="s">
@@ -1637,10 +1637,10 @@
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A42" s="14"/>
       <c r="B42" s="15"/>
       <c r="C42" s="3" t="s">
@@ -1650,10 +1650,10 @@
         <v>52</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A43" s="14"/>
       <c r="B43" s="15" t="s">
         <v>55</v>
@@ -1665,10 +1665,10 @@
         <v>54</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
       <c r="B44" s="15"/>
       <c r="C44" s="3" t="s">
@@ -1678,10 +1678,10 @@
         <v>57</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A45" s="14"/>
       <c r="B45" s="15"/>
       <c r="C45" s="3" t="s">
@@ -1691,10 +1691,10 @@
         <v>73</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="15"/>
       <c r="C46" s="3" t="s">
@@ -1704,10 +1704,10 @@
         <v>75</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A47" s="14"/>
       <c r="B47" s="15" t="s">
         <v>59</v>
@@ -1719,10 +1719,10 @@
         <v>76</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A48" s="14"/>
       <c r="B48" s="15"/>
       <c r="C48" s="3" t="s">
@@ -1732,10 +1732,10 @@
         <v>77</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A49" s="14"/>
       <c r="B49" s="15"/>
       <c r="C49" s="3" t="s">
@@ -1745,10 +1745,10 @@
         <v>78</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A50" s="14"/>
       <c r="B50" s="15"/>
       <c r="C50" s="3" t="s">
@@ -1758,10 +1758,10 @@
         <v>83</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A51" s="14"/>
       <c r="B51" s="15"/>
       <c r="C51" s="3" t="s">
@@ -1771,10 +1771,10 @@
         <v>79</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A52" s="14"/>
       <c r="B52" s="15"/>
       <c r="C52" s="3" t="s">
@@ -1784,7 +1784,7 @@
         <v>80</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>